<commit_message>
Update reports 2026-08-28 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-08-28.xlsx
+++ b/gex_pivot_levels_2026-08-28.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Pivots" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CL'!$A$1:$G$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -109,10 +109,10 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -544,12 +544,12 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>-$11.04M</t>
+          <t>-$17.35M</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+$21.98M</t>
+          <t>+$27.78M</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -560,44 +560,40 @@
       <c r="G2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="2" t="n">
         <v>7651.51</v>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="2" t="n">
         <v>7640</v>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>-$7.23M</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>+$11.57M</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>-$6.90M</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>+$11.05M</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>7656.51</v>
+        <v>7661.51</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>7645</v>
+        <v>7650</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -606,53 +602,49 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>-$1.89M</t>
+          <t>-$6.58M</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+$2.88M</t>
+          <t>+$14.65M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>7661.29</v>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>763</v>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="A5" s="5" t="n">
+        <v>7681.34</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>765</v>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>-$14.25M</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>+$22.93M</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>-$51.74M</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>+$91.28M</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -660,10 +652,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>7661.51</v>
+        <v>7686.51</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>7650</v>
+        <v>7675</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
@@ -672,12 +664,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>-$6.83M</t>
+          <t>-$1.90M</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>+$15.22M</t>
+          <t>+$18.99M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -689,24 +681,24 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>7681.34</v>
+        <v>7711.42</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>765</v>
+        <v>768</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>-$9.99M</t>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>+$32.68K</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>+$55.64M</t>
+          <t>+$102.54M</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -717,87 +709,87 @@
       <c r="G7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>7686.51</v>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>7675</v>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="A8" s="5" t="n">
+        <v>7711.51</v>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>7700</v>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>-$1.95M</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>+$19.43M</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>-$14.46M</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>+$59.48M</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>7731.47</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>770</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>+$35.41M</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>+$183.78M</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="n">
-        <v>7711.42</v>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>768</v>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>+$28.17M</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>+$62.67M</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="G9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>7711.51</v>
+        <v>7741.51</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>7700</v>
+        <v>7730</v>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>-$14.46M</t>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>+$16.63M</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>+$59.48M</t>
+          <t>+$35.75M</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -807,257 +799,257 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>7751.51</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>7740</v>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>+$4.14M</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>+$21.44M</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>7721.45</v>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>769</v>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>7751.52</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>772</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>+$9.98M</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>+$28.32M</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>+$47.46M</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>+$83.89M</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>7761.51</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>7750</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>+$11.23M</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>+$44.50M</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>7761.55</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>773</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>+$12.52M</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>+$36.13M</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="n">
-        <v>7731.47</v>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>770</v>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>7781.51</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>7770</v>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>+$19.33M</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>+$21.88M</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>7781.6</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>775</v>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>+$54.94M</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>+$118.97M</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>+$51.10M</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>+$66.94M</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="n">
-        <v>7741.51</v>
-      </c>
-      <c r="B13" s="5" t="n">
-        <v>7730</v>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>7806.51</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>7795</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>+$16.43M</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>+$35.31M</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="n">
-        <v>7751.51</v>
-      </c>
-      <c r="B14" s="5" t="n">
-        <v>7740</v>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>+$4.04M</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>+$20.92M</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>+$4.49M</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>+$5.05M</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>7761.51</v>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>7750</v>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>+$10.94M</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>+$43.37M</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>7761.55</v>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>773</v>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>+$5.85M</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>+$26.93M</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="n">
-        <v>7781.51</v>
-      </c>
-      <c r="B17" s="5" t="n">
-        <v>7770</v>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>+$18.70M</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>+$21.16M</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
-        <v>7781.6</v>
+        <v>7811.51</v>
       </c>
       <c r="B18" s="5" t="n">
-        <v>775</v>
+        <v>7800</v>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>+$32.81M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>+$14.82M</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>+$50.09M</t>
+          <t>+$19.59M</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1073,101 +1065,35 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>7806.51</v>
+        <v>7851.51</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>7795</v>
+        <v>7840</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>+$4.34M</t>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>+$5.75M</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>+$4.89M</t>
+          <t>+$5.83M</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="n">
-        <v>7811.51</v>
-      </c>
-      <c r="B20" s="5" t="n">
-        <v>7800</v>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>+$14.82M</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>+$19.59M</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>7851.51</v>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>7840</v>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>+$5.75M</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>+$5.83M</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr"/>
+      <c r="G19" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G21"/>
+  <autoFilter ref="A1:G19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1269,7 +1195,7 @@
           <t>QQQ</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>+$69.49K</t>
         </is>
@@ -1298,7 +1224,7 @@
           <t>QQQ</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>+$35.02M</t>
         </is>
@@ -1331,7 +1257,7 @@
           <t>QQQ</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>+$3.44M</t>
         </is>
@@ -1364,7 +1290,7 @@
           <t>NDX</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>+$322.80K</t>
         </is>
@@ -1393,7 +1319,7 @@
           <t>NDX</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>+$444.62K</t>
         </is>
@@ -1459,7 +1385,7 @@
           <t>NDX</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>+$2.69M</t>
         </is>
@@ -1492,7 +1418,7 @@
           <t>QQQ</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>+$12.49M</t>
         </is>
@@ -1521,7 +1447,7 @@
           <t>NDX</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>+$298.79K</t>
         </is>
@@ -1550,7 +1476,7 @@
           <t>QQQ</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>+$53.66M</t>
         </is>
@@ -1583,7 +1509,7 @@
           <t>NDX</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>+$240.69K</t>
         </is>
@@ -1645,7 +1571,7 @@
           <t>NDX</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>+$182.59K</t>
         </is>
@@ -1736,7 +1662,7 @@
           <t>NDX</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>+$215.79K</t>
         </is>
@@ -1765,7 +1691,7 @@
           <t>NDX</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t>+$2.51M</t>
         </is>
@@ -1798,7 +1724,7 @@
           <t>NDX</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>+$11.56K</t>
         </is>
@@ -1831,7 +1757,7 @@
           <t>NDX</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>+$455.29K</t>
         </is>
@@ -1860,7 +1786,7 @@
           <t>QQQ</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>+$27.91M</t>
         </is>
@@ -1893,7 +1819,7 @@
           <t>NDX</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>+$910.59K</t>
         </is>
@@ -1926,7 +1852,7 @@
           <t>QQQ</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>+$1.62M</t>
         </is>
@@ -1959,7 +1885,7 @@
           <t>QQQ</t>
         </is>
       </c>
-      <c r="D25" s="8" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>+$33.03M</t>
         </is>
@@ -1992,7 +1918,7 @@
           <t>QQQ</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
+      <c r="D26" s="8" t="inlineStr">
         <is>
           <t>+$8.54M</t>
         </is>
@@ -2182,7 +2108,7 @@
           <t>IWM</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>+$11.64M</t>
         </is>
@@ -2310,7 +2236,7 @@
           <t>USO</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>+$2.00M</t>
         </is>
@@ -2376,7 +2302,7 @@
           <t>USO</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>+$1.67M</t>
         </is>
@@ -2409,7 +2335,7 @@
           <t>USO</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>+$497.06K</t>
         </is>
@@ -2442,7 +2368,7 @@
           <t>USO</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>+$1.83M</t>
         </is>
@@ -2537,7 +2463,7 @@
           <t>GDX</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>+$1.33M</t>
         </is>
@@ -2595,7 +2521,7 @@
           <t>GLD</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>+$14.37M</t>
         </is>
@@ -2661,7 +2587,7 @@
           <t>GDX</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>+$41.57M</t>
         </is>
@@ -2694,7 +2620,7 @@
           <t>GLD</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>+$71.39M</t>
         </is>
@@ -2727,7 +2653,7 @@
           <t>GLD</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>+$11.16M</t>
         </is>
@@ -2756,7 +2682,7 @@
           <t>GDX</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>+$458.12K</t>
         </is>
@@ -2789,7 +2715,7 @@
           <t>GDX</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>+$16.14M</t>
         </is>
@@ -2822,7 +2748,7 @@
           <t>GLD</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>+$7.61M</t>
         </is>
@@ -2852,7 +2778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2908,106 +2834,98 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B2" s="5" t="n">
+      <c r="B2" s="2" t="n">
         <v>7731.47</v>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="2" t="n">
         <v>770</v>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>+$54.94M</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>+$118.97M</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>+$35.41M</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>+$183.78M</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n">
-        <v>29650.12</v>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>720</v>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>QQQ</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>7711.42</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>768</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>+$53.66M</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>+$83.15M</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>+$32.68K</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>+$102.54M</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>4636.38</v>
+        <v>7681.34</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>425</v>
+        <v>765</v>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>+$71.39M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>-$51.74M</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>+$79.81M</t>
+          <t>+$91.28M</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -3017,43 +2935,43 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
-        <v>7711.42</v>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>768</v>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="B5" s="2" t="n">
+        <v>7751.52</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>772</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>+$28.17M</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>+$62.67M</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
+          <t>+$47.46M</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>+$83.89M</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -3062,28 +2980,28 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>7711.51</v>
+        <v>29650.12</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>7700</v>
+        <v>720</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>-$14.46M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>+$53.66M</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>+$59.48M</t>
+          <t>+$83.15M</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -3093,35 +3011,35 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>29444.6</v>
+        <v>4636.38</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>715</v>
+        <v>425</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>+$35.02M</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>+$71.39M</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>+$55.84M</t>
+          <t>+$79.81M</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -3136,64 +3054,68 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
-        <v>7681.34</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>765</v>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="B8" s="5" t="n">
+        <v>7781.6</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>775</v>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>-$9.99M</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>+$55.64M</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr"/>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>+$51.10M</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>+$66.94M</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>3018</v>
+        <v>7711.51</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>300</v>
+        <v>7700</v>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>-$29.57M</t>
+          <t>-$14.46M</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>+$51.40M</t>
+          <t>+$59.48M</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -3210,28 +3132,28 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>7781.6</v>
+        <v>29444.6</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>775</v>
+        <v>715</v>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>+$32.81M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>+$35.02M</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>+$50.09M</t>
+          <t>+$55.84M</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -3248,112 +3170,112 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>3018</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>300</v>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>-$29.57M</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>+$51.40M</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B12" s="5" t="n">
         <v>4623.98</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C12" s="5" t="n">
         <v>104</v>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>+$41.57M</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>+$45.54M</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B13" s="2" t="n">
         <v>7761.51</v>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="C13" s="2" t="n">
         <v>7750</v>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>+$10.94M</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>+$43.37M</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>+$11.23M</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>+$44.50M</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="n">
-        <v>29855.65</v>
-      </c>
-      <c r="C13" s="5" t="n">
-        <v>725</v>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>+$27.91M</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>+$37.65M</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="H13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -3362,24 +3284,24 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>30061.18</v>
+        <v>29855.65</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>730</v>
+        <v>725</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>+$33.03M</t>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>+$27.91M</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>+$37.09M</t>
+          <t>+$37.65M</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -3396,188 +3318,188 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>30061.18</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>730</v>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>+$33.03M</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>+$37.09M</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
-        <v>7741.51</v>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>7730</v>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>+$16.43M</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>+$35.31M</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>4581.84</v>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>420</v>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
+      <c r="B16" s="2" t="n">
+        <v>7761.55</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>773</v>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>+$14.37M</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>+$32.64M</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
+          <t>+$12.52M</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>+$36.13M</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>7741.51</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>7730</v>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>+$16.63M</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>+$35.75M</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>4581.84</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>420</v>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>+$14.37M</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>+$32.64M</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
           <t>RTY</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B19" s="5" t="n">
         <v>2967.7</v>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C19" s="5" t="n">
         <v>295</v>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>-$31.37M</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>+$32.63M</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>7721.45</v>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>769</v>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>+$9.98M</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>+$28.32M</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>29691.23</v>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>721</v>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>-$10.44M</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>+$27.27M</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -3590,36 +3512,32 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>7761.55</v>
+        <v>7631.21</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>773</v>
+        <v>760</v>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>+$5.85M</t>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>-$17.35M</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>+$26.93M</t>
+          <t>+$27.78M</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -3628,70 +3546,70 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>29567.91</v>
+        <v>29691.23</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>718</v>
+        <v>721</v>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>+$12.49M</t>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>-$10.44M</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>+$25.21M</t>
+          <t>+$27.27M</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>7661.29</v>
+        <v>29567.91</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>763</v>
+        <v>718</v>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>-$14.25M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>+$12.49M</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>+$22.93M</t>
+          <t>+$25.21M</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -3710,7 +3628,7 @@
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>+$69.49K</t>
         </is>
@@ -3728,38 +3646,42 @@
       <c r="H23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
-        <v>7631.21</v>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>760</v>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>-$11.04M</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>+$21.98M</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr"/>
+      <c r="B24" s="5" t="n">
+        <v>7781.51</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>7770</v>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>+$19.33M</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>+$21.88M</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -3768,24 +3690,24 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>7781.51</v>
+        <v>7751.51</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>7770</v>
+        <v>7740</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>+$18.70M</t>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>+$4.14M</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>+$21.16M</t>
+          <t>+$21.44M</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
@@ -3795,7 +3717,7 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -3806,24 +3728,24 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>7751.51</v>
+        <v>7811.51</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>7740</v>
+        <v>7800</v>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>+$4.04M</t>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>+$14.82M</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>+$20.92M</t>
+          <t>+$19.59M</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
@@ -3833,107 +3755,107 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B27" s="5" t="n">
-        <v>7811.51</v>
-      </c>
-      <c r="C27" s="5" t="n">
-        <v>7800</v>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="B27" s="2" t="n">
+        <v>7686.51</v>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>7675</v>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>+$14.82M</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>+$19.59M</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>-$1.90M</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>+$18.99M</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>3048.18</v>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>303</v>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>+$11.64M</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>+$16.94M</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="n">
-        <v>7686.51</v>
-      </c>
-      <c r="C28" s="2" t="n">
-        <v>7675</v>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>-$1.95M</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>+$19.43M</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>3048.18</v>
+        <v>4757.37</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>303</v>
+        <v>107</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E29" s="8" t="inlineStr">
-        <is>
-          <t>+$11.64M</t>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>+$16.14M</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>+$16.94M</t>
+          <t>+$16.15M</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -3948,68 +3870,64 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="n">
-        <v>4757.37</v>
-      </c>
-      <c r="C30" s="5" t="n">
-        <v>107</v>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>+$16.14M</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>+$16.15M</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>7661.51</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>7650</v>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>-$6.58M</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>+$14.65M</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>7661.51</v>
+        <v>4690.93</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>7650</v>
+        <v>430</v>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>-$6.83M</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>+$11.16M</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>+$15.22M</t>
+          <t>+$12.92M</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -4022,28 +3940,28 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>4690.93</v>
+        <v>7651.51</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>430</v>
+        <v>7640</v>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E32" s="9" t="inlineStr">
-        <is>
-          <t>+$11.16M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>-$6.90M</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>+$12.92M</t>
+          <t>+$11.05M</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -4054,68 +3972,64 @@
       <c r="H32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="n">
-        <v>7651.51</v>
-      </c>
-      <c r="C33" s="5" t="n">
-        <v>7640</v>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>-$7.23M</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
-        <is>
-          <t>+$11.57M</t>
-        </is>
-      </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>29033.54</v>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>705</v>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>-$4.94M</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>+$10.33M</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>29033.54</v>
+        <v>4446.14</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>705</v>
+        <v>100</v>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>-$4.94M</t>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>+$1.33M</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>+$10.33M</t>
+          <t>+$9.52M</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -4132,24 +4046,24 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>4446.14</v>
+        <v>4516.38</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>100</v>
+        <v>414</v>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E35" s="9" t="inlineStr">
-        <is>
-          <t>+$1.33M</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>-$7.95M</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>+$9.52M</t>
+          <t>+$8.96M</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -4162,28 +4076,28 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>4516.38</v>
+        <v>30266.71</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>414</v>
+        <v>735</v>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>-$7.95M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>+$8.54M</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>+$8.96M</t>
+          <t>+$8.54M</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
@@ -4200,202 +4114,206 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>30266.71</v>
+        <v>29485.7</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>735</v>
+        <v>716</v>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E37" s="9" t="inlineStr">
-        <is>
-          <t>+$8.54M</t>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>+$3.44M</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>+$8.54M</t>
+          <t>+$8.33M</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>29485.7</v>
+        <v>4800.02</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>716</v>
+        <v>440</v>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E38" s="9" t="inlineStr">
-        <is>
-          <t>+$3.44M</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>+$7.61M</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>+$8.33M</t>
+          <t>+$7.66M</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>85.81999999999999</v>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>130</v>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>-$1.99M</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>+$6.06M</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="n">
-        <v>4800.02</v>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>440</v>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E39" s="9" t="inlineStr">
-        <is>
-          <t>+$7.61M</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>+$7.66M</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>7851.51</v>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>7840</v>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>+$5.75M</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>+$5.83M</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="n">
-        <v>85.81999999999999</v>
-      </c>
-      <c r="C40" s="5" t="n">
-        <v>130</v>
-      </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="inlineStr">
-        <is>
-          <t>-$1.99M</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="inlineStr">
-        <is>
-          <t>+$6.06M</t>
-        </is>
-      </c>
-      <c r="G40" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H40" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>7851.51</v>
+        <v>2977.76</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>7840</v>
+        <v>296</v>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E41" s="9" t="inlineStr">
-        <is>
-          <t>+$5.75M</t>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>-$4.03M</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>+$5.83M</t>
+          <t>+$5.69M</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>2977.76</v>
+        <v>7806.51</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>296</v>
+        <v>7795</v>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>-$4.03M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>+$4.49M</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>+$5.69M</t>
+          <t>+$5.05M</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -4405,35 +4323,35 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>7806.51</v>
+        <v>85.16</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>7795</v>
+        <v>129</v>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E43" s="9" t="inlineStr">
-        <is>
-          <t>+$4.34M</t>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>+$2.00M</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>+$4.89M</t>
+          <t>+$3.24M</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -4443,157 +4361,157 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>29554.19</v>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>29500</v>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>+$2.69M</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>+$3.14M</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="n">
+        <v>4614.56</v>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>423</v>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>-$185.88K</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>+$3.07M</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B44" s="2" t="n">
-        <v>85.16</v>
-      </c>
-      <c r="C44" s="2" t="n">
-        <v>129</v>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
+      <c r="B46" s="5" t="n">
+        <v>89.12</v>
+      </c>
+      <c r="C46" s="5" t="n">
+        <v>135</v>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E44" s="9" t="inlineStr">
-        <is>
-          <t>+$2.00M</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>+$3.24M</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H44" s="3" t="inlineStr">
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>+$1.83M</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>+$2.69M</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="6" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B45" s="5" t="n">
-        <v>29554.19</v>
-      </c>
-      <c r="C45" s="5" t="n">
-        <v>29500</v>
-      </c>
-      <c r="D45" s="6" t="inlineStr">
+      <c r="B47" s="5" t="n">
+        <v>29814.19</v>
+      </c>
+      <c r="C47" s="5" t="n">
+        <v>29760</v>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>+$2.69M</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
-          <t>+$3.14M</t>
-        </is>
-      </c>
-      <c r="G45" s="6" t="inlineStr">
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>+$2.51M</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>+$2.51M</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H45" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="n">
-        <v>4614.56</v>
-      </c>
-      <c r="C46" s="2" t="n">
-        <v>423</v>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>-$185.88K</t>
-        </is>
-      </c>
-      <c r="F46" s="3" t="inlineStr">
-        <is>
-          <t>+$3.07M</t>
-        </is>
-      </c>
-      <c r="G46" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H46" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="n">
-        <v>7656.51</v>
-      </c>
-      <c r="C47" s="2" t="n">
-        <v>7645</v>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>-$1.89M</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="inlineStr">
-        <is>
-          <t>+$2.88M</t>
-        </is>
-      </c>
-      <c r="G47" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H47" s="3" t="inlineStr">
+      <c r="H47" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4606,24 +4524,24 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>89.12</v>
+        <v>87.14</v>
       </c>
       <c r="C48" s="5" t="n">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>+$1.83M</t>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>+$1.67M</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>+$2.69M</t>
+          <t>+$2.48M</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
@@ -4640,104 +4558,104 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>82.52</v>
+      </c>
+      <c r="C49" s="5" t="n">
+        <v>125</v>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>-$1.54M</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>+$2.09M</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B49" s="5" t="n">
-        <v>29814.19</v>
-      </c>
-      <c r="C49" s="5" t="n">
-        <v>29760</v>
-      </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>+$2.51M</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="inlineStr">
-        <is>
-          <t>+$2.51M</t>
-        </is>
-      </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H49" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="n">
-        <v>87.14</v>
-      </c>
-      <c r="C50" s="5" t="n">
-        <v>132</v>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>USO</t>
+      <c r="B50" s="2" t="n">
+        <v>29958.41</v>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>727.5</v>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t>+$1.67M</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>+$2.48M</t>
-        </is>
-      </c>
-      <c r="G50" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H50" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
+          <t>+$1.62M</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>+$1.83M</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>82.52</v>
+        <v>29879.19</v>
       </c>
       <c r="C51" s="5" t="n">
-        <v>125</v>
+        <v>29825</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="inlineStr">
-        <is>
-          <t>-$1.54M</t>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E51" s="9" t="inlineStr">
+        <is>
+          <t>+$910.59K</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>+$2.09M</t>
+          <t>+$910.59K</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
@@ -4747,35 +4665,35 @@
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>29958.41</v>
+        <v>4712.91</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>727.5</v>
+        <v>106</v>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E52" s="9" t="inlineStr">
-        <is>
-          <t>+$1.62M</t>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>+$458.12K</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>+$1.83M</t>
+          <t>+$833.33K</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
@@ -4790,152 +4708,148 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="n">
-        <v>29879.19</v>
-      </c>
-      <c r="C53" s="5" t="n">
-        <v>29825</v>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>88.45999999999999</v>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t>+$910.59K</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>+$910.59K</t>
-        </is>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H53" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
+          <t>+$497.06K</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>+$660.97K</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>4712.91</v>
+        <v>29854.19</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>106</v>
+        <v>29800</v>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E54" s="9" t="inlineStr">
-        <is>
-          <t>+$458.12K</t>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>+$455.29K</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>+$833.33K</t>
+          <t>+$618.92K</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>88.45999999999999</v>
+        <v>29504.19</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>134</v>
+        <v>29450</v>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E55" s="9" t="inlineStr">
-        <is>
-          <t>+$497.06K</t>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>+$322.80K</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>+$660.97K</t>
+          <t>+$570.60K</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H55" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B56" s="2" t="n">
-        <v>29854.19</v>
-      </c>
-      <c r="C56" s="2" t="n">
-        <v>29800</v>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="B56" s="5" t="n">
+        <v>29524.19</v>
+      </c>
+      <c r="C56" s="5" t="n">
+        <v>29470</v>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>+$455.29K</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="inlineStr">
-        <is>
-          <t>+$618.92K</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H56" s="3" t="inlineStr"/>
+          <t>+$444.62K</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>+$451.74K</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -4944,24 +4858,24 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>29504.19</v>
+        <v>29654.19</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>29450</v>
+        <v>29600</v>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E57" s="9" t="inlineStr">
-        <is>
-          <t>+$322.80K</t>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>+$240.69K</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>+$570.60K</t>
+          <t>+$373.48K</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
@@ -4972,42 +4886,38 @@
       <c r="H57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="inlineStr">
+      <c r="A58" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B58" s="5" t="n">
-        <v>29524.19</v>
-      </c>
-      <c r="C58" s="5" t="n">
-        <v>29470</v>
-      </c>
-      <c r="D58" s="6" t="inlineStr">
+      <c r="B58" s="2" t="n">
+        <v>29629.19</v>
+      </c>
+      <c r="C58" s="2" t="n">
+        <v>29575</v>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
         <is>
-          <t>+$444.62K</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="inlineStr">
-        <is>
-          <t>+$451.74K</t>
-        </is>
-      </c>
-      <c r="G58" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H58" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>+$298.79K</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>+$356.88K</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -5016,24 +4926,24 @@
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>29654.19</v>
+        <v>29704.19</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>29600</v>
+        <v>29650</v>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E59" s="9" t="inlineStr">
-        <is>
-          <t>+$240.69K</t>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>+$182.59K</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>+$373.48K</t>
+          <t>+$348.58K</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
@@ -5050,24 +4960,24 @@
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>29629.19</v>
+        <v>29724.19</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>29575</v>
+        <v>29670</v>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E60" s="9" t="inlineStr">
-        <is>
-          <t>+$298.79K</t>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>-$215.79K</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>+$356.88K</t>
+          <t>+$307.09K</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
@@ -5084,32 +4994,36 @@
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>29704.19</v>
+        <v>29729.19</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>29650</v>
+        <v>29675</v>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E61" s="9" t="inlineStr">
-        <is>
-          <t>+$182.59K</t>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>-$219.94K</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>+$348.58K</t>
+          <t>+$286.34K</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H61" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -5118,24 +5032,24 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>29724.19</v>
+        <v>29754.19</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>29670</v>
+        <v>29700</v>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E62" s="4" t="inlineStr">
-        <is>
-          <t>-$215.79K</t>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>+$215.79K</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>+$307.09K</t>
+          <t>+$273.89K</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
@@ -5152,10 +5066,10 @@
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>29729.19</v>
+        <v>29534.19</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>29675</v>
+        <v>29480</v>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
@@ -5164,12 +5078,12 @@
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>-$219.94K</t>
+          <t>-$67.58K</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>+$286.34K</t>
+          <t>+$88.92K</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -5190,111 +5104,39 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>29754.19</v>
+        <v>29834.19</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>29700</v>
+        <v>29780</v>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E64" s="9" t="inlineStr">
-        <is>
-          <t>+$215.79K</t>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>+$11.56K</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>+$273.89K</t>
+          <t>+$11.56K</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H64" s="3" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="n">
-        <v>29534.19</v>
-      </c>
-      <c r="C65" s="2" t="n">
-        <v>29480</v>
-      </c>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E65" s="4" t="inlineStr">
-        <is>
-          <t>-$67.58K</t>
-        </is>
-      </c>
-      <c r="F65" s="3" t="inlineStr">
-        <is>
-          <t>+$88.92K</t>
-        </is>
-      </c>
-      <c r="G65" s="3" t="inlineStr">
-        <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H65" s="3" t="inlineStr">
+      <c r="H64" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="n">
-        <v>29834.19</v>
-      </c>
-      <c r="C66" s="2" t="n">
-        <v>29780</v>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E66" s="9" t="inlineStr">
-        <is>
-          <t>+$11.56K</t>
-        </is>
-      </c>
-      <c r="F66" s="3" t="inlineStr">
-        <is>
-          <t>+$11.56K</t>
-        </is>
-      </c>
-      <c r="G66" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H66" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H66"/>
+  <autoFilter ref="A1:H64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>